<commit_message>
fix: adjust password regex
</commit_message>
<xml_diff>
--- a/Casos_de_Teste_Agroscope_Completo.xlsx
+++ b/Casos_de_Teste_Agroscope_Completo.xlsx
@@ -685,7 +685,7 @@
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Senha: senha@123</t>
+          <t>Senha: Senha@123</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>3. Preencher o campo de senha com senha@123 → Campo exibe os caracteres mascarados</t>
+          <t>3. Preencher o campo de senha com Senha@123 → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F5" s="7" t="n"/>
@@ -777,7 +777,7 @@
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Senha: senha@123</t>
+          <t>Senha: Senha@123</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -796,7 +796,7 @@
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>3. Preencher o campo de senha com senha@123 → Campo exibe os caracteres mascarados</t>
+          <t>3. Preencher o campo de senha com Senha@123 → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F9" s="7" t="n"/>
@@ -1053,7 +1053,7 @@
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Senha: qualquerSenha@123</t>
+          <t>Senha: QualquerSenha@123</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -1072,7 +1072,7 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>3. Preencher o campo de senha com qualquerSenha@123 → Campo exibe os caracteres mascarados</t>
+          <t>3. Preencher o campo de senha com QualquerSenha@123 → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F21" s="7" t="n"/>
@@ -1433,12 +1433,12 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Nova senha: novaSenha@456</t>
+          <t>Nova senha: NovaSenha@456</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>1. Na tela de nova senha, digitar novaSenha@456 no campo de nova senha → Campo exibe os caracteres mascarados</t>
+          <t>1. Na tela de nova senha, digitar NovaSenha@456 no campo de nova senha → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -1468,7 +1468,7 @@
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>2. Digitar novaSenha@456 no campo de confirmação → Campo exibe os caracteres mascarados</t>
+          <t>2. Digitar NovaSenha@456 no campo de confirmação → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F37" s="7" t="n"/>
@@ -1711,7 +1711,7 @@
       <c r="C47" s="7" t="n"/>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Senha: senha@123</t>
+          <t>Senha: Senha@123</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -1730,7 +1730,7 @@
       <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>4. Preencher o campo de senha com senha@123 → Campo exibe os caracteres mascarados</t>
+          <t>4. Preencher o campo de senha com Senha@123 → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F48" s="7" t="n"/>
@@ -1835,7 +1835,7 @@
       <c r="C53" s="7" t="n"/>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Senha: outraSenha@123</t>
+          <t>Senha: OutraSenha@123</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -1995,7 +1995,7 @@
       <c r="C59" s="7" t="n"/>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Senha: senha@123</t>
+          <t>Senha: Senha@123</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -2014,7 +2014,7 @@
       <c r="D60" s="7" t="n"/>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>4. Preencher o campo de senha com senha@123 → Campo exibe os caracteres mascarados</t>
+          <t>4. Preencher o campo de senha com Senha@123 → Campo exibe os caracteres mascarados</t>
         </is>
       </c>
       <c r="F60" s="7" t="n"/>

</xml_diff>

<commit_message>
feat: update test cases spreadsheet
</commit_message>
<xml_diff>
--- a/Casos_de_Teste_Agroscope_Completo.xlsx
+++ b/Casos_de_Teste_Agroscope_Completo.xlsx
@@ -203,6 +203,47 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00000000"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFD966"/>
+          <bgColor rgb="00FFD966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0070AD47"/>
+          <bgColor rgb="0070AD47"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C00000"/>
+          <bgColor rgb="00C00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -3687,6 +3728,22 @@
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H63:H66"/>
   </mergeCells>
+  <conditionalFormatting sqref="H2:H300">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pendente"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Aprovado"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Reprovado"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Pendente,Aprovado,Reprovado"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>